<commit_message>
Updated IND model - 2025-09-12 15:56
</commit_message>
<xml_diff>
--- a/VerveStacks_IND/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_IND/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_IND\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{031D0189-49EB-4FFF-A3D2-95267C367B66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F76482F8-A82C-49CC-85D2-8CBF68D7F219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -979,34 +979,34 @@
     <t>solar resource -- CF class spv-IND_16 -- cost class 4</t>
   </si>
   <si>
+    <t>e_spv-IND_0_c5</t>
+  </si>
+  <si>
+    <t>solar resource -- CF class spv-IND_0 -- cost class 5</t>
+  </si>
+  <si>
+    <t>e_spv-IND_0_c2</t>
+  </si>
+  <si>
+    <t>solar resource -- CF class spv-IND_0 -- cost class 2</t>
+  </si>
+  <si>
+    <t>e_spv-IND_0_c1</t>
+  </si>
+  <si>
+    <t>solar resource -- CF class spv-IND_0 -- cost class 1</t>
+  </si>
+  <si>
     <t>e_spv-IND_0_c3</t>
   </si>
   <si>
     <t>solar resource -- CF class spv-IND_0 -- cost class 3</t>
   </si>
   <si>
-    <t>e_spv-IND_0_c1</t>
-  </si>
-  <si>
-    <t>solar resource -- CF class spv-IND_0 -- cost class 1</t>
-  </si>
-  <si>
     <t>e_spv-IND_0_c4</t>
   </si>
   <si>
     <t>solar resource -- CF class spv-IND_0 -- cost class 4</t>
-  </si>
-  <si>
-    <t>e_spv-IND_0_c5</t>
-  </si>
-  <si>
-    <t>solar resource -- CF class spv-IND_0 -- cost class 5</t>
-  </si>
-  <si>
-    <t>e_spv-IND_0_c2</t>
-  </si>
-  <si>
-    <t>solar resource -- CF class spv-IND_0 -- cost class 2</t>
   </si>
   <si>
     <t>comm-out</t>
@@ -7950,7 +7950,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAE42652-1440-4710-B690-CA44501A8F26}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3A33852-C79D-4A74-9686-786AEBE80038}">
   <dimension ref="B9:N64"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9891,13 +9891,13 @@
         <v>297</v>
       </c>
       <c r="L60">
-        <v>0.77364403067522491</v>
+        <v>5.2500000000000003E-3</v>
       </c>
       <c r="M60">
         <v>0</v>
       </c>
       <c r="N60">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="61" spans="2:14">
@@ -9929,13 +9929,13 @@
         <v>297</v>
       </c>
       <c r="L61">
-        <v>3.2726001779475915</v>
+        <v>5.3282119260176248</v>
       </c>
       <c r="M61">
         <v>0</v>
       </c>
       <c r="N61">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="62" spans="2:14">
@@ -9967,13 +9967,13 @@
         <v>297</v>
       </c>
       <c r="L62">
-        <v>4.4778378857750975E-2</v>
+        <v>3.2726001779475915</v>
       </c>
       <c r="M62">
         <v>0</v>
       </c>
       <c r="N62">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63" spans="2:14">
@@ -10005,13 +10005,13 @@
         <v>297</v>
       </c>
       <c r="L63">
-        <v>5.2500000000000003E-3</v>
+        <v>0.77364403067522491</v>
       </c>
       <c r="M63">
         <v>0</v>
       </c>
       <c r="N63">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="64" spans="2:14">
@@ -10043,13 +10043,13 @@
         <v>297</v>
       </c>
       <c r="L64">
-        <v>5.3282119260176248</v>
+        <v>4.4778378857750975E-2</v>
       </c>
       <c r="M64">
         <v>0</v>
       </c>
       <c r="N64">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -10058,7 +10058,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BD131F0-1802-4537-848C-C6BD234EBE9B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A41D5BEC-9FC1-41AA-9D97-9CCDCF1CDEE5}">
   <dimension ref="B9:AB219"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -22490,7 +22490,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9B2E44C-662D-422E-85C4-4E37EBB6A084}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F588028C-2F7B-45D9-8674-918C54C9EE71}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated IND model - 2025-09-12 16:01
</commit_message>
<xml_diff>
--- a/VerveStacks_IND/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_IND/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_IND\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F76482F8-A82C-49CC-85D2-8CBF68D7F219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3DAC02A2-2084-40C5-8FE0-D62B067D3B65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -979,6 +979,12 @@
     <t>solar resource -- CF class spv-IND_16 -- cost class 4</t>
   </si>
   <si>
+    <t>e_spv-IND_0_c1</t>
+  </si>
+  <si>
+    <t>solar resource -- CF class spv-IND_0 -- cost class 1</t>
+  </si>
+  <si>
     <t>e_spv-IND_0_c5</t>
   </si>
   <si>
@@ -989,12 +995,6 @@
   </si>
   <si>
     <t>solar resource -- CF class spv-IND_0 -- cost class 2</t>
-  </si>
-  <si>
-    <t>e_spv-IND_0_c1</t>
-  </si>
-  <si>
-    <t>solar resource -- CF class spv-IND_0 -- cost class 1</t>
   </si>
   <si>
     <t>e_spv-IND_0_c3</t>
@@ -7950,7 +7950,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3A33852-C79D-4A74-9686-786AEBE80038}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5004431C-2AE8-4E45-940C-8EC85C3C166F}">
   <dimension ref="B9:N64"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9891,13 +9891,13 @@
         <v>297</v>
       </c>
       <c r="L60">
-        <v>5.2500000000000003E-3</v>
+        <v>3.2726001779475915</v>
       </c>
       <c r="M60">
         <v>0</v>
       </c>
       <c r="N60">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61" spans="2:14">
@@ -9929,13 +9929,13 @@
         <v>297</v>
       </c>
       <c r="L61">
-        <v>5.3282119260176248</v>
+        <v>5.2500000000000003E-3</v>
       </c>
       <c r="M61">
         <v>0</v>
       </c>
       <c r="N61">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="62" spans="2:14">
@@ -9967,13 +9967,13 @@
         <v>297</v>
       </c>
       <c r="L62">
-        <v>3.2726001779475915</v>
+        <v>5.3282119260176248</v>
       </c>
       <c r="M62">
         <v>0</v>
       </c>
       <c r="N62">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="63" spans="2:14">
@@ -10058,7 +10058,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A41D5BEC-9FC1-41AA-9D97-9CCDCF1CDEE5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26A5721E-0D5F-4C2D-B180-1B46C55EF90C}">
   <dimension ref="B9:AB219"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -22490,7 +22490,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F588028C-2F7B-45D9-8674-918C54C9EE71}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4F77C4C-A962-46D0-A458-DA32111059A7}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN model - 2025-09-13 01:37
</commit_message>
<xml_diff>
--- a/VerveStacks_IND/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_IND/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_IND\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3DAC02A2-2084-40C5-8FE0-D62B067D3B65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E2F70220-2914-4988-BEC0-72D2F16B26B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -979,34 +979,34 @@
     <t>solar resource -- CF class spv-IND_16 -- cost class 4</t>
   </si>
   <si>
+    <t>e_spv-IND_0_c2</t>
+  </si>
+  <si>
+    <t>solar resource -- CF class spv-IND_0 -- cost class 2</t>
+  </si>
+  <si>
+    <t>e_spv-IND_0_c3</t>
+  </si>
+  <si>
+    <t>solar resource -- CF class spv-IND_0 -- cost class 3</t>
+  </si>
+  <si>
     <t>e_spv-IND_0_c1</t>
   </si>
   <si>
     <t>solar resource -- CF class spv-IND_0 -- cost class 1</t>
   </si>
   <si>
+    <t>e_spv-IND_0_c4</t>
+  </si>
+  <si>
+    <t>solar resource -- CF class spv-IND_0 -- cost class 4</t>
+  </si>
+  <si>
     <t>e_spv-IND_0_c5</t>
   </si>
   <si>
     <t>solar resource -- CF class spv-IND_0 -- cost class 5</t>
-  </si>
-  <si>
-    <t>e_spv-IND_0_c2</t>
-  </si>
-  <si>
-    <t>solar resource -- CF class spv-IND_0 -- cost class 2</t>
-  </si>
-  <si>
-    <t>e_spv-IND_0_c3</t>
-  </si>
-  <si>
-    <t>solar resource -- CF class spv-IND_0 -- cost class 3</t>
-  </si>
-  <si>
-    <t>e_spv-IND_0_c4</t>
-  </si>
-  <si>
-    <t>solar resource -- CF class spv-IND_0 -- cost class 4</t>
   </si>
   <si>
     <t>comm-out</t>
@@ -7950,7 +7950,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5004431C-2AE8-4E45-940C-8EC85C3C166F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01B04CBC-D2F7-444D-8528-01CE92E6E380}">
   <dimension ref="B9:N64"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9891,13 +9891,13 @@
         <v>297</v>
       </c>
       <c r="L60">
-        <v>3.2726001779475915</v>
+        <v>5.3282119260176248</v>
       </c>
       <c r="M60">
         <v>0</v>
       </c>
       <c r="N60">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="61" spans="2:14">
@@ -9929,13 +9929,13 @@
         <v>297</v>
       </c>
       <c r="L61">
-        <v>5.2500000000000003E-3</v>
+        <v>0.77364403067522491</v>
       </c>
       <c r="M61">
         <v>0</v>
       </c>
       <c r="N61">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="62" spans="2:14">
@@ -9967,13 +9967,13 @@
         <v>297</v>
       </c>
       <c r="L62">
-        <v>5.3282119260176248</v>
+        <v>3.2726001779475915</v>
       </c>
       <c r="M62">
         <v>0</v>
       </c>
       <c r="N62">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63" spans="2:14">
@@ -10005,13 +10005,13 @@
         <v>297</v>
       </c>
       <c r="L63">
-        <v>0.77364403067522491</v>
+        <v>4.4778378857750975E-2</v>
       </c>
       <c r="M63">
         <v>0</v>
       </c>
       <c r="N63">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="64" spans="2:14">
@@ -10043,13 +10043,13 @@
         <v>297</v>
       </c>
       <c r="L64">
-        <v>4.4778378857750975E-2</v>
+        <v>5.2500000000000003E-3</v>
       </c>
       <c r="M64">
         <v>0</v>
       </c>
       <c r="N64">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -10058,7 +10058,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26A5721E-0D5F-4C2D-B180-1B46C55EF90C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65FDD5A5-A00E-4D2B-9FFA-68AEFC2D1BA3}">
   <dimension ref="B9:AB219"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -22490,7 +22490,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4F77C4C-A962-46D0-A458-DA32111059A7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{567932EE-9D4A-48C3-89FD-083F1952C802}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated IND model - 2025-09-13 01:45
</commit_message>
<xml_diff>
--- a/VerveStacks_IND/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_IND/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_IND\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E2F70220-2914-4988-BEC0-72D2F16B26B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{91C669C6-B10F-466B-AF7E-15EBB01CFAAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -979,6 +979,18 @@
     <t>solar resource -- CF class spv-IND_16 -- cost class 4</t>
   </si>
   <si>
+    <t>e_spv-IND_0_c5</t>
+  </si>
+  <si>
+    <t>solar resource -- CF class spv-IND_0 -- cost class 5</t>
+  </si>
+  <si>
+    <t>e_spv-IND_0_c1</t>
+  </si>
+  <si>
+    <t>solar resource -- CF class spv-IND_0 -- cost class 1</t>
+  </si>
+  <si>
     <t>e_spv-IND_0_c2</t>
   </si>
   <si>
@@ -991,22 +1003,10 @@
     <t>solar resource -- CF class spv-IND_0 -- cost class 3</t>
   </si>
   <si>
-    <t>e_spv-IND_0_c1</t>
-  </si>
-  <si>
-    <t>solar resource -- CF class spv-IND_0 -- cost class 1</t>
-  </si>
-  <si>
     <t>e_spv-IND_0_c4</t>
   </si>
   <si>
     <t>solar resource -- CF class spv-IND_0 -- cost class 4</t>
-  </si>
-  <si>
-    <t>e_spv-IND_0_c5</t>
-  </si>
-  <si>
-    <t>solar resource -- CF class spv-IND_0 -- cost class 5</t>
   </si>
   <si>
     <t>comm-out</t>
@@ -7950,7 +7950,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01B04CBC-D2F7-444D-8528-01CE92E6E380}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B32914F-268D-4591-BE85-95323F3E4F06}">
   <dimension ref="B9:N64"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9891,13 +9891,13 @@
         <v>297</v>
       </c>
       <c r="L60">
-        <v>5.3282119260176248</v>
+        <v>5.2500000000000003E-3</v>
       </c>
       <c r="M60">
         <v>0</v>
       </c>
       <c r="N60">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="61" spans="2:14">
@@ -9929,13 +9929,13 @@
         <v>297</v>
       </c>
       <c r="L61">
-        <v>0.77364403067522491</v>
+        <v>3.2726001779475915</v>
       </c>
       <c r="M61">
         <v>0</v>
       </c>
       <c r="N61">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="62" spans="2:14">
@@ -9967,13 +9967,13 @@
         <v>297</v>
       </c>
       <c r="L62">
-        <v>3.2726001779475915</v>
+        <v>5.3282119260176248</v>
       </c>
       <c r="M62">
         <v>0</v>
       </c>
       <c r="N62">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="63" spans="2:14">
@@ -10005,13 +10005,13 @@
         <v>297</v>
       </c>
       <c r="L63">
-        <v>4.4778378857750975E-2</v>
+        <v>0.77364403067522491</v>
       </c>
       <c r="M63">
         <v>0</v>
       </c>
       <c r="N63">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="64" spans="2:14">
@@ -10043,13 +10043,13 @@
         <v>297</v>
       </c>
       <c r="L64">
-        <v>5.2500000000000003E-3</v>
+        <v>4.4778378857750975E-2</v>
       </c>
       <c r="M64">
         <v>0</v>
       </c>
       <c r="N64">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -10058,7 +10058,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65FDD5A5-A00E-4D2B-9FFA-68AEFC2D1BA3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D59CA7D7-36B7-494E-83FE-3A07D89ADEAE}">
   <dimension ref="B9:AB219"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -22490,7 +22490,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{567932EE-9D4A-48C3-89FD-083F1952C802}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D288BBC1-6B0B-4A32-B1B3-12CEA2941353}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated IND model - 2025-09-13 09:07
</commit_message>
<xml_diff>
--- a/VerveStacks_IND/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_IND/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_IND\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{91C669C6-B10F-466B-AF7E-15EBB01CFAAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3D17198F-CFFA-4CB1-A4FA-638DCA5E1A93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -979,6 +979,18 @@
     <t>solar resource -- CF class spv-IND_16 -- cost class 4</t>
   </si>
   <si>
+    <t>e_spv-IND_0_c2</t>
+  </si>
+  <si>
+    <t>solar resource -- CF class spv-IND_0 -- cost class 2</t>
+  </si>
+  <si>
+    <t>e_spv-IND_0_c4</t>
+  </si>
+  <si>
+    <t>solar resource -- CF class spv-IND_0 -- cost class 4</t>
+  </si>
+  <si>
     <t>e_spv-IND_0_c5</t>
   </si>
   <si>
@@ -991,22 +1003,10 @@
     <t>solar resource -- CF class spv-IND_0 -- cost class 1</t>
   </si>
   <si>
-    <t>e_spv-IND_0_c2</t>
-  </si>
-  <si>
-    <t>solar resource -- CF class spv-IND_0 -- cost class 2</t>
-  </si>
-  <si>
     <t>e_spv-IND_0_c3</t>
   </si>
   <si>
     <t>solar resource -- CF class spv-IND_0 -- cost class 3</t>
-  </si>
-  <si>
-    <t>e_spv-IND_0_c4</t>
-  </si>
-  <si>
-    <t>solar resource -- CF class spv-IND_0 -- cost class 4</t>
   </si>
   <si>
     <t>comm-out</t>
@@ -7950,7 +7950,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B32914F-268D-4591-BE85-95323F3E4F06}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D3DB30B-2552-4D72-A327-35228E516C70}">
   <dimension ref="B9:N64"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9891,13 +9891,13 @@
         <v>297</v>
       </c>
       <c r="L60">
-        <v>5.2500000000000003E-3</v>
+        <v>5.3282119260176248</v>
       </c>
       <c r="M60">
         <v>0</v>
       </c>
       <c r="N60">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="61" spans="2:14">
@@ -9929,13 +9929,13 @@
         <v>297</v>
       </c>
       <c r="L61">
-        <v>3.2726001779475915</v>
+        <v>4.4778378857750975E-2</v>
       </c>
       <c r="M61">
         <v>0</v>
       </c>
       <c r="N61">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="62" spans="2:14">
@@ -9967,13 +9967,13 @@
         <v>297</v>
       </c>
       <c r="L62">
-        <v>5.3282119260176248</v>
+        <v>5.2500000000000003E-3</v>
       </c>
       <c r="M62">
         <v>0</v>
       </c>
       <c r="N62">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="63" spans="2:14">
@@ -10005,13 +10005,13 @@
         <v>297</v>
       </c>
       <c r="L63">
-        <v>0.77364403067522491</v>
+        <v>3.2726001779475915</v>
       </c>
       <c r="M63">
         <v>0</v>
       </c>
       <c r="N63">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64" spans="2:14">
@@ -10043,13 +10043,13 @@
         <v>297</v>
       </c>
       <c r="L64">
-        <v>4.4778378857750975E-2</v>
+        <v>0.77364403067522491</v>
       </c>
       <c r="M64">
         <v>0</v>
       </c>
       <c r="N64">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -10058,7 +10058,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D59CA7D7-36B7-494E-83FE-3A07D89ADEAE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9E06FEC-01C7-4C1E-B1A8-465436E350A5}">
   <dimension ref="B9:AB219"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -22490,7 +22490,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D288BBC1-6B0B-4A32-B1B3-12CEA2941353}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E3CE1D0-0606-479C-A9D2-D5527A2F367F}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated IND model - 2025-09-13 09:49
</commit_message>
<xml_diff>
--- a/VerveStacks_IND/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_IND/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_IND\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3D17198F-CFFA-4CB1-A4FA-638DCA5E1A93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9E1837F8-3CB9-4CC2-9428-D97A5072FD39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -979,34 +979,34 @@
     <t>solar resource -- CF class spv-IND_16 -- cost class 4</t>
   </si>
   <si>
+    <t>e_spv-IND_0_c1</t>
+  </si>
+  <si>
+    <t>solar resource -- CF class spv-IND_0 -- cost class 1</t>
+  </si>
+  <si>
+    <t>e_spv-IND_0_c3</t>
+  </si>
+  <si>
+    <t>solar resource -- CF class spv-IND_0 -- cost class 3</t>
+  </si>
+  <si>
+    <t>e_spv-IND_0_c5</t>
+  </si>
+  <si>
+    <t>solar resource -- CF class spv-IND_0 -- cost class 5</t>
+  </si>
+  <si>
+    <t>e_spv-IND_0_c4</t>
+  </si>
+  <si>
+    <t>solar resource -- CF class spv-IND_0 -- cost class 4</t>
+  </si>
+  <si>
     <t>e_spv-IND_0_c2</t>
   </si>
   <si>
     <t>solar resource -- CF class spv-IND_0 -- cost class 2</t>
-  </si>
-  <si>
-    <t>e_spv-IND_0_c4</t>
-  </si>
-  <si>
-    <t>solar resource -- CF class spv-IND_0 -- cost class 4</t>
-  </si>
-  <si>
-    <t>e_spv-IND_0_c5</t>
-  </si>
-  <si>
-    <t>solar resource -- CF class spv-IND_0 -- cost class 5</t>
-  </si>
-  <si>
-    <t>e_spv-IND_0_c1</t>
-  </si>
-  <si>
-    <t>solar resource -- CF class spv-IND_0 -- cost class 1</t>
-  </si>
-  <si>
-    <t>e_spv-IND_0_c3</t>
-  </si>
-  <si>
-    <t>solar resource -- CF class spv-IND_0 -- cost class 3</t>
   </si>
   <si>
     <t>comm-out</t>
@@ -7950,7 +7950,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D3DB30B-2552-4D72-A327-35228E516C70}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{111F68D9-CD61-461F-8069-AA54A5CA7695}">
   <dimension ref="B9:N64"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9891,13 +9891,13 @@
         <v>297</v>
       </c>
       <c r="L60">
-        <v>5.3282119260176248</v>
+        <v>3.2726001779475915</v>
       </c>
       <c r="M60">
         <v>0</v>
       </c>
       <c r="N60">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61" spans="2:14">
@@ -9929,13 +9929,13 @@
         <v>297</v>
       </c>
       <c r="L61">
-        <v>4.4778378857750975E-2</v>
+        <v>0.77364403067522491</v>
       </c>
       <c r="M61">
         <v>0</v>
       </c>
       <c r="N61">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="62" spans="2:14">
@@ -10005,13 +10005,13 @@
         <v>297</v>
       </c>
       <c r="L63">
-        <v>3.2726001779475915</v>
+        <v>4.4778378857750975E-2</v>
       </c>
       <c r="M63">
         <v>0</v>
       </c>
       <c r="N63">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="64" spans="2:14">
@@ -10043,13 +10043,13 @@
         <v>297</v>
       </c>
       <c r="L64">
-        <v>0.77364403067522491</v>
+        <v>5.3282119260176248</v>
       </c>
       <c r="M64">
         <v>0</v>
       </c>
       <c r="N64">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -10058,7 +10058,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9E06FEC-01C7-4C1E-B1A8-465436E350A5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8434CE1D-7DB1-4727-92F0-5DEAA8071B1F}">
   <dimension ref="B9:AB219"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -22490,7 +22490,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E3CE1D0-0606-479C-A9D2-D5527A2F367F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D855002-F526-4F56-96F4-F72BE6D1AF89}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated IND model - 2025-09-14 18:03
</commit_message>
<xml_diff>
--- a/VerveStacks_IND/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_IND/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_IND\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9E1837F8-3CB9-4CC2-9428-D97A5072FD39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{44FC1C4C-C609-4EC5-B48A-7E0320C9A247}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -985,16 +985,16 @@
     <t>solar resource -- CF class spv-IND_0 -- cost class 1</t>
   </si>
   <si>
+    <t>e_spv-IND_0_c5</t>
+  </si>
+  <si>
+    <t>solar resource -- CF class spv-IND_0 -- cost class 5</t>
+  </si>
+  <si>
     <t>e_spv-IND_0_c3</t>
   </si>
   <si>
     <t>solar resource -- CF class spv-IND_0 -- cost class 3</t>
-  </si>
-  <si>
-    <t>e_spv-IND_0_c5</t>
-  </si>
-  <si>
-    <t>solar resource -- CF class spv-IND_0 -- cost class 5</t>
   </si>
   <si>
     <t>e_spv-IND_0_c4</t>
@@ -7950,7 +7950,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{111F68D9-CD61-461F-8069-AA54A5CA7695}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C225FDC7-0641-4A47-A973-3FCD4D0BB948}">
   <dimension ref="B9:N64"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -9929,13 +9929,13 @@
         <v>297</v>
       </c>
       <c r="L61">
-        <v>0.77364403067522491</v>
+        <v>5.2500000000000003E-3</v>
       </c>
       <c r="M61">
         <v>0</v>
       </c>
       <c r="N61">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="62" spans="2:14">
@@ -9967,13 +9967,13 @@
         <v>297</v>
       </c>
       <c r="L62">
-        <v>5.2500000000000003E-3</v>
+        <v>0.77364403067522491</v>
       </c>
       <c r="M62">
         <v>0</v>
       </c>
       <c r="N62">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="63" spans="2:14">
@@ -10058,7 +10058,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8434CE1D-7DB1-4727-92F0-5DEAA8071B1F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA4F1ABE-1914-4A1B-80C9-12DE77C254E0}">
   <dimension ref="B9:AB219"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -22490,7 +22490,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D855002-F526-4F56-96F4-F72BE6D1AF89}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00FAC20D-4FED-43E8-A04B-C7117D731F6B}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>